<commit_message>
Task 3: event impact modeling with S-curve function and validation
</commit_message>
<xml_diff>
--- a/data/raw/ethiopia_fi_unified_data.xlsx
+++ b/data/raw/ethiopia_fi_unified_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ethiopia_fi_unified_data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Impact_sheet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ethiopia_fi_unified_data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact_sheet" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH50"/>
+  <dimension ref="A1:AH52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5655,7 +5655,7 @@
       </c>
       <c r="AH48" t="inlineStr">
         <is>
-          <t>Recomputed 57% male - 42% female = 15pp. Supersedes REC_0028's medium-confidence 18pp estimate; retain both and flag the discrepancy in EDA.</t>
+          <t>Recomputed 57% male - 42% female = 15pp.</t>
         </is>
       </c>
     </row>
@@ -5771,7 +5771,7 @@
       </c>
       <c r="AH49" t="inlineStr">
         <is>
-          <t>New indicator: share of adults with accounts usable for card/phone/app payments. Highlights the access-vs-usage gap central to this challenge.</t>
+          <t>New indicator: digitally enabled accounts</t>
         </is>
       </c>
     </row>
@@ -5876,12 +5876,244 @@
       </c>
       <c r="AG50" t="inlineStr">
         <is>
-          <t>the Ethiopian Parliament approved the new Banking Business law, which allows foreign banks and foreigners to rejoin the Ethiopian market after an absence of half a century</t>
+          <t>the Ethiopian Parliament approved the new Banking Business law</t>
         </is>
       </c>
       <c r="AH50" t="inlineStr">
         <is>
-          <t>NBE began accepting foreign bank license applications June 25, 2025. First major banking-sector liberalization event; not yet captured in dataset.</t>
+          <t>Banking-sector liberalization event</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>REC_0039</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>observation</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>USAGE</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Digital Payment Adoption Rate</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>USG_DIGITAL_PAYMENT</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>higher_better</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>20</v>
+      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2021-06-30</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="n">
+        <v>2021</v>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>national</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>World Bank Blog (Global Findex 2021)</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>https://blogs.worldbank.org/en/africacan/mobile-phone-technology-could-expand-equitable-access-financial-services-ethiopia</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr"/>
+      <c r="X51" t="inlineStr"/>
+      <c r="Y51" t="inlineStr"/>
+      <c r="Z51" t="inlineStr"/>
+      <c r="AA51" t="inlineStr"/>
+      <c r="AB51" t="inlineStr"/>
+      <c r="AC51" t="inlineStr"/>
+      <c r="AD51" t="inlineStr"/>
+      <c r="AE51" t="inlineStr">
+        <is>
+          <t>Betel Yohannes</t>
+        </is>
+      </c>
+      <c r="AF51" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="AG51" t="inlineStr">
+        <is>
+          <t>Only 42 percent of account holders—20 percent of adults—used their accounts for digital payments in the year prior to the Global Findex survey</t>
+        </is>
+      </c>
+      <c r="AH51" t="inlineStr">
+        <is>
+          <t>Critical gap fix: this is the actual Usage pillar target (Digital Payment Adoption Rate) the assignment asks us to forecast, previously entirely absent from the dataset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>REC_0040</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>observation</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>USAGE</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Digital Payment Adoption Rate</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>USG_DIGITAL_PAYMENT</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>higher_better</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>35</v>
+      </c>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2024-11-29</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="n">
+        <v>2024</v>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>national</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Global Findex 2024 (per challenge brief)</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>survey</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>challenge brief: Forecasting Financial Inclusion in Ethiopia (Overview section)</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr"/>
+      <c r="X52" t="inlineStr"/>
+      <c r="Y52" t="inlineStr"/>
+      <c r="Z52" t="inlineStr"/>
+      <c r="AA52" t="inlineStr"/>
+      <c r="AB52" t="inlineStr"/>
+      <c r="AC52" t="inlineStr"/>
+      <c r="AD52" t="inlineStr"/>
+      <c r="AE52" t="inlineStr">
+        <is>
+          <t>Betel Yohannes</t>
+        </is>
+      </c>
+      <c r="AF52" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="AG52" t="inlineStr">
+        <is>
+          <t>Made or received digital payment: ~35%</t>
+        </is>
+      </c>
+      <c r="AH52" t="inlineStr">
+        <is>
+          <t>Figure provided directly in the assignment brief. Note: a Shega/DFS Ethiopia Hub article describes digital payments as used by 'fewer than one in four adults' (~24%) in 2024 -- a discrepancy from the brief's ~35%, likely reflecting different question wording or survey rounds. The brief's figure is used since it is the explicit forecasting target for this project; the discrepancy is flagged as a data quality caveat.</t>
         </is>
       </c>
     </row>
@@ -7799,7 +8031,7 @@
       <c r="AH16" t="inlineStr"/>
       <c r="AI16" t="inlineStr">
         <is>
-          <t>Foreign capital/competition effects on retail account ownership are typically slow; too recent for empirical Ethiopian data.</t>
+          <t>Foreign capital/competition effects are slow</t>
         </is>
       </c>
     </row>
@@ -7896,7 +8128,7 @@
       <c r="AH17" t="inlineStr"/>
       <c r="AI17" t="inlineStr">
         <is>
-          <t>NFIS-II (2021) previously had no modeled impact_link despite being the umbrella policy with the 70%-by-2025 target. National strategies commonly undershoot targets; flagged as uncertain.</t>
+          <t>NFIS-II umbrella policy, previously unlinked</t>
         </is>
       </c>
     </row>

</xml_diff>